<commit_message>
reran a bunch of fecundity analyses
</commit_message>
<xml_diff>
--- a/raw_data/mass_data.xlsx
+++ b/raw_data/mass_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joegunn/Desktop/Projects/active_projects/CPB_Phenotype/raw_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6EC4A90-0E3A-144B-B58E-3A5E34A4A3A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86A086E6-7116-5845-97C6-47C93A21A6A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1560" windowWidth="25600" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="16400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3490,7 +3490,7 @@
         <v>L5_F0_E</v>
       </c>
       <c r="F84" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G84" s="4" t="s">
         <v>44</v>
@@ -3526,7 +3526,7 @@
         <v>L5_F0_E</v>
       </c>
       <c r="F85" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G85" s="4" t="s">
         <v>44</v>
@@ -3562,7 +3562,7 @@
         <v>L5_F0_E</v>
       </c>
       <c r="F86" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G86" s="4" t="s">
         <v>44</v>
@@ -3596,7 +3596,7 @@
         <v>L5_F0_E</v>
       </c>
       <c r="F87" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G87" s="4" t="s">
         <v>44</v>
@@ -3630,7 +3630,7 @@
         <v>L7_F0_C</v>
       </c>
       <c r="F88" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G88" s="4" t="s">
         <v>44</v>
@@ -3664,7 +3664,7 @@
         <v>L7_F0_C</v>
       </c>
       <c r="F89" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G89" s="4" t="s">
         <v>44</v>
@@ -3698,7 +3698,7 @@
         <v>L8_F0_C</v>
       </c>
       <c r="F90" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G90" s="4" t="s">
         <v>44</v>
@@ -3734,7 +3734,7 @@
         <v>L8_F0_C</v>
       </c>
       <c r="F91" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G91" s="4" t="s">
         <v>44</v>
@@ -3770,7 +3770,7 @@
         <v>L8_F0_E</v>
       </c>
       <c r="F92" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G92" s="4" t="s">
         <v>44</v>
@@ -3804,7 +3804,7 @@
         <v>L8_F0_E</v>
       </c>
       <c r="F93" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G93" s="4" t="s">
         <v>44</v>
@@ -3838,7 +3838,7 @@
         <v>L10_F0_C</v>
       </c>
       <c r="F94" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G94" s="4" t="s">
         <v>44</v>
@@ -3874,7 +3874,7 @@
         <v>L10_F0_C</v>
       </c>
       <c r="F95" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G95" s="4" t="s">
         <v>44</v>
@@ -3910,7 +3910,7 @@
         <v>L10_F0_C</v>
       </c>
       <c r="F96" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G96" s="4" t="s">
         <v>44</v>
@@ -3944,7 +3944,7 @@
         <v>L10_F0_C</v>
       </c>
       <c r="F97" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G97" s="4" t="s">
         <v>44</v>
@@ -3978,7 +3978,7 @@
         <v>L11_F0_C</v>
       </c>
       <c r="F98" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G98" s="4" t="s">
         <v>44</v>
@@ -4014,7 +4014,7 @@
         <v>L11_F0_C</v>
       </c>
       <c r="F99" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G99" s="4" t="s">
         <v>44</v>
@@ -4050,7 +4050,7 @@
         <v>L1_F0_C</v>
       </c>
       <c r="F100" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G100" s="4" t="s">
         <v>13</v>
@@ -4084,7 +4084,7 @@
         <v>L1_F0_C</v>
       </c>
       <c r="F101" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G101" s="4" t="s">
         <v>13</v>
@@ -4118,7 +4118,7 @@
         <v>L1_F0_E</v>
       </c>
       <c r="F102" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G102" s="4" t="s">
         <v>13</v>
@@ -4154,7 +4154,7 @@
         <v>L1_F0_E</v>
       </c>
       <c r="F103" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G103" s="4" t="s">
         <v>13</v>
@@ -4190,7 +4190,7 @@
         <v>L1_F0_E</v>
       </c>
       <c r="F104" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G104" s="4" t="s">
         <v>13</v>
@@ -4224,7 +4224,7 @@
         <v>L1_F0_E</v>
       </c>
       <c r="F105" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G105" s="4" t="s">
         <v>13</v>
@@ -4258,7 +4258,7 @@
         <v>L3_F0_C</v>
       </c>
       <c r="F106" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G106" s="4" t="s">
         <v>13</v>
@@ -4292,7 +4292,7 @@
         <v>L3_F0_C</v>
       </c>
       <c r="F107" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G107" s="4" t="s">
         <v>13</v>
@@ -4326,7 +4326,7 @@
         <v>L4_F0_C</v>
       </c>
       <c r="F108" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G108" s="4" t="s">
         <v>13</v>
@@ -4360,7 +4360,7 @@
         <v>L4_F0_C</v>
       </c>
       <c r="F109" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G109" s="4" t="s">
         <v>13</v>
@@ -4394,7 +4394,7 @@
         <v>L4_F0_C</v>
       </c>
       <c r="F110" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G110" s="4" t="s">
         <v>13</v>
@@ -4428,7 +4428,7 @@
         <v>L4_F0_C</v>
       </c>
       <c r="F111" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G111" s="4" t="s">
         <v>13</v>
@@ -4462,7 +4462,7 @@
         <v>L4_F0_C</v>
       </c>
       <c r="F112" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G112" s="4" t="s">
         <v>13</v>
@@ -4496,7 +4496,7 @@
         <v>L4_F0_C</v>
       </c>
       <c r="F113" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G113" s="4" t="s">
         <v>13</v>
@@ -4530,7 +4530,7 @@
         <v>L5_F0_C</v>
       </c>
       <c r="F114" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G114" s="4" t="s">
         <v>13</v>
@@ -4564,7 +4564,7 @@
         <v>L5_F0_C</v>
       </c>
       <c r="F115" s="5">
-        <v>46106</v>
+        <v>45376</v>
       </c>
       <c r="G115" s="4" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
added summary data analyses for founder egg data
</commit_message>
<xml_diff>
--- a/raw_data/mass_data.xlsx
+++ b/raw_data/mass_data.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joegunn/Desktop/Projects/active_projects/CPB_Phenotype/raw_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joegunn/Desktop/projects/active_projects/CPB_Phenotype/raw_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F30EB5D7-CB4B-5944-962D-A7823F43904B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D4369E4-7397-5843-94FD-A1411C620BA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="280" yWindow="1740" windowWidth="25040" windowHeight="16940" xr2:uid="{F6EF0537-9742-074D-B090-2FBA022A3466}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -670,6 +670,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD83DECA-8B26-844E-BE88-B5260C4BEAC5}">
   <dimension ref="A1:K668"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="10" max="10" width="22.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">

</xml_diff>